<commit_message>
Update IT APP teaching spreadsheets
Refreshes the Excel-based teaching materials for the IT APP course by updating the lesson and intermediate spreadsheet files used in the training set.
</commit_message>
<xml_diff>
--- a/Teorie/2.IT/APP/prostredni.xlsx
+++ b/Teorie/2.IT/APP/prostredni.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scmsd-my.sharepoint.com/personal/it-martinsramek_stredniskola_com/Documents/Plocha/SCMSD-IT-Martin-Sramek/Teorie/2.IT/APP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{1617A1F7-E5F2-4A57-AFF4-984077686C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{271579B0-A7C5-485C-977D-2E207B2B0401}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="8_{1617A1F7-E5F2-4A57-AFF4-984077686C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FBEFDF6-4357-4234-9CEB-7F9FCAF634EA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{160D8B57-2C18-44C7-918E-3A066D99840C}"/>
   </bookViews>
@@ -3143,7 +3143,125 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>311729</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>138547</xdr:colOff>
+      <xdr:row>119</xdr:row>
+      <xdr:rowOff>41237</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Obrázek 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3748239-6A21-B1AA-E67E-86AC94C553BD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2130138" y="18669001"/>
+          <a:ext cx="7100454" cy="4041736"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>372718</xdr:colOff>
+      <xdr:row>119</xdr:row>
+      <xdr:rowOff>182217</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>8283</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="TextovéPole 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{000EBC79-17EF-29D2-6B82-CC0BC7A0E462}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2211457" y="22851717"/>
+          <a:ext cx="6982239" cy="1159566"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="cs-CZ" sz="1600"/>
+            <a:t>karta domu je rozdeelena na skupiny nastroji schranka pismo zarovani cislvoy styly bunk y</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3467,6 +3585,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add and update APP Excel workbooks
Adds two new Excel files (`EXCEL VYUKA.xlsx` and `priklady2.xlsx`) and updates `prostredni.xlsx` under `Teorie/2.IT/APP`, expanding and refreshing the APP course spreadsheet materials.
</commit_message>
<xml_diff>
--- a/Teorie/2.IT/APP/prostredni.xlsx
+++ b/Teorie/2.IT/APP/prostredni.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scmsd-my.sharepoint.com/personal/it-martinsramek_stredniskola_com/Documents/Plocha/SCMSD-IT-Martin-Sramek/Teorie/2.IT/APP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="134" documentId="8_{1617A1F7-E5F2-4A57-AFF4-984077686C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42555392-3289-4794-98F8-71F1046D7004}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{1617A1F7-E5F2-4A57-AFF4-984077686C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{375B0DA9-59B3-4A32-A68F-7A2547F533D0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{160D8B57-2C18-44C7-918E-3A066D99840C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{160D8B57-2C18-44C7-918E-3A066D99840C}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
+    <sheet name="List2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3707,4 +3708,13 @@
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D292EBA7-E121-4FFD-84AB-FBDB9036FB8D}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>